<commit_message>
Compact workbook column widths
</commit_message>
<xml_diff>
--- a/downloads/part-time-efficiency/20260706-20260712/panda-part-time-efficiency-weekend-holidays.xlsx
+++ b/downloads/part-time-efficiency/20260706-20260712/panda-part-time-efficiency-weekend-holidays.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="老板总览" sheetId="1" r:id="R29c3e3a4f5da4cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="门店周数据录入" sheetId="2" r:id="R8f011e71f477434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则参数" sheetId="3" r:id="R1253bb6e6d294ee9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="引流周汇总" sheetId="4" r:id="R2626f9de7b454ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复位周汇总" sheetId="5" r:id="Rfeba62da540a461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据校验" sheetId="6" r:id="R7806ec96959b488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店长每日填写模板" sheetId="7" r:id="R391de2d816364d9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="8" r:id="R6719c8ddc83647eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="老板总览" sheetId="1" r:id="R369e49cc573c4921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="门店周数据录入" sheetId="2" r:id="Ref24323e1d154461"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则参数" sheetId="3" r:id="R30df9e309c3f450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="引流周汇总" sheetId="4" r:id="Rc1f5ad98fde84e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复位周汇总" sheetId="5" r:id="R3814360c489942eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据校验" sheetId="6" r:id="R6845c33ce2044c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店长每日填写模板" sheetId="7" r:id="R57e294b2b23c47c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="8" r:id="Rbb47ad2382b94502"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -273,14 +273,6 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
@@ -288,6 +280,14 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1646,24 +1646,24 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="31.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="8" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="8.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="8.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="6.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1934,7 +1934,7 @@
         <x:f>'引流周汇总'!R4</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="K10" s="38" t="str">
+      <x:c r="K10" s="34" t="str">
         <x:f>'引流周汇总'!T4</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
@@ -2008,7 +2008,7 @@
         <x:f>'引流周汇总'!R5</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="K11" s="39" t="str">
+      <x:c r="K11" s="35" t="str">
         <x:f>'引流周汇总'!T5</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
@@ -2082,7 +2082,7 @@
         <x:f>'引流周汇总'!R6</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="K12" s="39" t="str">
+      <x:c r="K12" s="35" t="str">
         <x:f>'引流周汇总'!T6</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
@@ -2156,7 +2156,7 @@
         <x:f>'引流周汇总'!R7</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K13" s="39" t="str">
+      <x:c r="K13" s="35" t="str">
         <x:f>'引流周汇总'!T7</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2230,7 +2230,7 @@
         <x:f>'引流周汇总'!R8</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K14" s="39" t="str">
+      <x:c r="K14" s="35" t="str">
         <x:f>'引流周汇总'!T8</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2304,7 +2304,7 @@
         <x:f>'引流周汇总'!R9</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="K15" s="39" t="str">
+      <x:c r="K15" s="35" t="str">
         <x:f>'引流周汇总'!T9</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
@@ -2378,7 +2378,7 @@
         <x:f>'引流周汇总'!R10</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="K16" s="39" t="str">
+      <x:c r="K16" s="35" t="str">
         <x:f>'引流周汇总'!T10</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
@@ -2452,7 +2452,7 @@
         <x:f>'引流周汇总'!R11</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K17" s="39" t="str">
+      <x:c r="K17" s="35" t="str">
         <x:f>'引流周汇总'!T11</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2526,7 +2526,7 @@
         <x:f>'引流周汇总'!R12</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K18" s="39" t="str">
+      <x:c r="K18" s="35" t="str">
         <x:f>'引流周汇总'!T12</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2600,7 +2600,7 @@
         <x:f>'引流周汇总'!R13</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K19" s="39" t="str">
+      <x:c r="K19" s="35" t="str">
         <x:f>'引流周汇总'!T13</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2674,7 +2674,7 @@
         <x:f>'引流周汇总'!R14</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="K20" s="39" t="str">
+      <x:c r="K20" s="35" t="str">
         <x:f>'引流周汇总'!T14</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
@@ -2748,7 +2748,7 @@
         <x:f>'引流周汇总'!R15</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K21" s="39" t="str">
+      <x:c r="K21" s="35" t="str">
         <x:f>'引流周汇总'!T15</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2822,7 +2822,7 @@
         <x:f>'引流周汇总'!R16</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K22" s="39" t="str">
+      <x:c r="K22" s="35" t="str">
         <x:f>'引流周汇总'!T16</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2896,7 +2896,7 @@
         <x:f>'引流周汇总'!R17</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K23" s="39" t="str">
+      <x:c r="K23" s="35" t="str">
         <x:f>'引流周汇总'!T17</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -2970,7 +2970,7 @@
         <x:f>'引流周汇总'!R18</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="K24" s="39" t="str">
+      <x:c r="K24" s="35" t="str">
         <x:f>'引流周汇总'!T18</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
@@ -3044,7 +3044,7 @@
         <x:f>'引流周汇总'!R19</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K25" s="39" t="str">
+      <x:c r="K25" s="35" t="str">
         <x:f>'引流周汇总'!T19</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -3118,7 +3118,7 @@
         <x:f>'引流周汇总'!R20</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K26" s="39" t="str">
+      <x:c r="K26" s="35" t="str">
         <x:f>'引流周汇总'!T20</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -3192,7 +3192,7 @@
         <x:f>'引流周汇总'!R21</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="K27" s="39" t="str">
+      <x:c r="K27" s="35" t="str">
         <x:f>'引流周汇总'!T21</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
@@ -3265,7 +3265,7 @@
         <x:f>'引流周汇总'!R22</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="K28" s="40" t="str">
+      <x:c r="K28" s="36" t="str">
         <x:f>'引流周汇总'!T22</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
@@ -3358,7 +3358,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bc13e379e514ae5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0befb62cd3b44f13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3367,26 +3367,26 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="7.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.440000057220459" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="10" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="15" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="6.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="6.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="8.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="10" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="10.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="8.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="11.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="24.440000534057617" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -3414,28 +3414,28 @@
       <x:c r="T1" s="4"/>
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
-      <x:c r="A2" s="37" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>周期：2026-07-06至2026-07-12。引流只统计周六、周日及国家法定节假日；复位波次为周六、周日14:00-20:00。空白=缺失，0=业务确认确实为0。引流实际人工成本默认按工时×实际时薪+额外提成/奖励；源表复位工资周期尚待确认。</x:v>
       </x:c>
-      <x:c r="B2" s="37"/>
-      <x:c r="C2" s="37"/>
-      <x:c r="D2" s="37"/>
-      <x:c r="E2" s="37"/>
-      <x:c r="F2" s="37"/>
-      <x:c r="G2" s="37"/>
-      <x:c r="H2" s="37"/>
-      <x:c r="I2" s="37"/>
-      <x:c r="J2" s="37"/>
-      <x:c r="K2" s="37"/>
-      <x:c r="L2" s="37"/>
-      <x:c r="M2" s="37"/>
-      <x:c r="N2" s="37"/>
-      <x:c r="O2" s="37"/>
-      <x:c r="P2" s="37"/>
-      <x:c r="Q2" s="37"/>
-      <x:c r="R2" s="37"/>
-      <x:c r="S2" s="37"/>
-      <x:c r="T2" s="37"/>
+      <x:c r="B2" s="40"/>
+      <x:c r="C2" s="40"/>
+      <x:c r="D2" s="40"/>
+      <x:c r="E2" s="40"/>
+      <x:c r="F2" s="40"/>
+      <x:c r="G2" s="40"/>
+      <x:c r="H2" s="40"/>
+      <x:c r="I2" s="40"/>
+      <x:c r="J2" s="40"/>
+      <x:c r="K2" s="40"/>
+      <x:c r="L2" s="40"/>
+      <x:c r="M2" s="40"/>
+      <x:c r="N2" s="40"/>
+      <x:c r="O2" s="40"/>
+      <x:c r="P2" s="40"/>
+      <x:c r="Q2" s="40"/>
+      <x:c r="R2" s="40"/>
+      <x:c r="S2" s="40"/>
+      <x:c r="T2" s="40"/>
     </x:row>
     <x:row r="3" ht="34.5" customHeight="1">
       <x:c r="A3" s="16" t="str">
@@ -3556,7 +3556,7 @@
         <x:v>1833</x:v>
       </x:c>
       <x:c r="T4" s="41" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
@@ -3616,7 +3616,7 @@
         <x:v>2201</x:v>
       </x:c>
       <x:c r="T5" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="27" customHeight="1">
@@ -3676,7 +3676,7 @@
         <x:v>449</x:v>
       </x:c>
       <x:c r="T6" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
@@ -3736,7 +3736,7 @@
         <x:v>1967</x:v>
       </x:c>
       <x:c r="T7" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="27" customHeight="1">
@@ -3796,7 +3796,7 @@
         <x:v>2052</x:v>
       </x:c>
       <x:c r="T8" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="27" customHeight="1">
@@ -3856,7 +3856,7 @@
         <x:v>304</x:v>
       </x:c>
       <x:c r="T9" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="27" customHeight="1">
@@ -3916,7 +3916,7 @@
         <x:v>1809</x:v>
       </x:c>
       <x:c r="T10" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
@@ -3976,7 +3976,7 @@
         <x:v>1158</x:v>
       </x:c>
       <x:c r="T11" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
@@ -4036,7 +4036,7 @@
         <x:v>521</x:v>
       </x:c>
       <x:c r="T12" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
@@ -4096,7 +4096,7 @@
         <x:v>965</x:v>
       </x:c>
       <x:c r="T13" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
@@ -4156,7 +4156,7 @@
         <x:v>1504</x:v>
       </x:c>
       <x:c r="T14" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
@@ -4216,7 +4216,7 @@
         <x:v>1815</x:v>
       </x:c>
       <x:c r="T15" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
@@ -4276,7 +4276,7 @@
         <x:v>2629</x:v>
       </x:c>
       <x:c r="T16" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="27" customHeight="1">
@@ -4336,7 +4336,7 @@
         <x:v>1774</x:v>
       </x:c>
       <x:c r="T17" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="27" customHeight="1">
@@ -4396,7 +4396,7 @@
         <x:v>796</x:v>
       </x:c>
       <x:c r="T18" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="27" customHeight="1">
@@ -4456,7 +4456,7 @@
         <x:v>2005</x:v>
       </x:c>
       <x:c r="T19" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="27" customHeight="1">
@@ -4516,7 +4516,7 @@
         <x:v>281</x:v>
       </x:c>
       <x:c r="T20" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="27" customHeight="1">
@@ -4576,7 +4576,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="T21" s="42" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="27" customHeight="1">
@@ -4636,7 +4636,7 @@
         <x:v>1546</x:v>
       </x:c>
       <x:c r="T22" s="43" t="str">
-        <x:v>现值继承老板版，需确认已按周末/国家节假日过滤；到店/办卡待补</x:v>
+        <x:v>核对引流日期；补到店/办卡</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4654,7 +4654,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1fd60708f1840ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2e876a2c49f45bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4663,12 +4663,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="57.779998779296875" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="7.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="44.439998626708984" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -4692,234 +4692,234 @@
         <x:v>说明</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="23" t="str">
         <x:v>高峰小时数/天</x:v>
       </x:c>
       <x:c r="B4" s="26" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C4" s="23" t="str">
+      <x:c r="C4" s="34" t="str">
         <x:v>本版复位高峰为14:00-20:00</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="24" t="str">
         <x:v>高峰天数</x:v>
       </x:c>
       <x:c r="B5" s="27" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C5" s="24" t="str">
+      <x:c r="C5" s="35" t="str">
         <x:v>周六+周日，共12小时</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="24" t="str">
         <x:v>单主题平均游玩分钟</x:v>
       </x:c>
       <x:c r="B6" s="27" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C6" s="24" t="str">
+      <x:c r="C6" s="35" t="str">
         <x:v>只用于理论满负荷容量，不替代实际波次</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="24" t="str">
         <x:v>引流产出倍数低效线</x:v>
       </x:c>
       <x:c r="B7" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C7" s="24" t="str">
+      <x:c r="C7" s="35" t="str">
         <x:v>成交金额÷实际人工成本；它不是财务ROI</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="24" t="str">
         <x:v>引流产出倍数观察线</x:v>
       </x:c>
       <x:c r="B8" s="27" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C8" s="24" t="str">
+      <x:c r="C8" s="35" t="str">
         <x:v>低于10但不低于8进入观察</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="24" t="str">
         <x:v>每小时成交金额低效线</x:v>
       </x:c>
       <x:c r="B9" s="27" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C9" s="24" t="str">
+      <x:c r="C9" s="35" t="str">
         <x:v>低于此值优先检查点位、时段和排班</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="24" t="str">
         <x:v>引流工资率偏高线</x:v>
       </x:c>
       <x:c r="B10" s="29" t="n">
         <x:v>0.08</x:v>
       </x:c>
-      <x:c r="C10" s="24" t="str">
+      <x:c r="C10" s="35" t="str">
         <x:v>引流实际人工成本÷门店总营收</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="24" t="str">
         <x:v>同时负责主题下限</x:v>
       </x:c>
       <x:c r="B11" s="27" t="n">
         <x:v>2.5</x:v>
       </x:c>
-      <x:c r="C11" s="24" t="str">
+      <x:c r="C11" s="35" t="str">
         <x:v>低于且实际波次偏低，复位可能偏松</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:v>同时负责主题上限</x:v>
       </x:c>
       <x:c r="B12" s="27" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C12" s="24" t="str">
+      <x:c r="C12" s="35" t="str">
         <x:v>高于则存在结构性偏紧风险</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="24" t="str">
         <x:v>理论波次/人/时下限</x:v>
       </x:c>
       <x:c r="B13" s="27" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C13" s="24" t="str">
+      <x:c r="C13" s="35" t="str">
         <x:v>只作结构参考</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="24" t="str">
         <x:v>理论波次/人/时上限</x:v>
       </x:c>
       <x:c r="B14" s="27" t="n">
         <x:v>7.5</x:v>
       </x:c>
-      <x:c r="C14" s="24" t="str">
+      <x:c r="C14" s="35" t="str">
         <x:v>只作结构参考</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="24" t="str">
         <x:v>实际波次/人/时偏低线</x:v>
       </x:c>
       <x:c r="B15" s="27" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C15" s="24" t="str">
+      <x:c r="C15" s="35" t="str">
         <x:v>按两天12小时计算</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>实际波次/人/时偏高线</x:v>
       </x:c>
       <x:c r="B16" s="27" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C16" s="24" t="str">
+      <x:c r="C16" s="35" t="str">
         <x:v>按两天12小时计算</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="24" t="str">
         <x:v>高峰利用率偏紧线</x:v>
       </x:c>
       <x:c r="B17" s="29" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C17" s="24" t="str">
+      <x:c r="C17" s="35" t="str">
         <x:v>实际波次÷理论最大容量</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="24" t="str">
         <x:v>标准时薪</x:v>
       </x:c>
       <x:c r="B18" s="27" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C18" s="24" t="str">
+      <x:c r="C18" s="35" t="str">
         <x:v>横向比较、长期趋势统一使用</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="24" t="str">
         <x:v>连续验证周数</x:v>
       </x:c>
       <x:c r="B19" s="27" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C19" s="24" t="str">
+      <x:c r="C19" s="35" t="str">
         <x:v>禁止用单周数据直接淘汰人员</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="24" t="str">
         <x:v>创建人=实际接待负责人</x:v>
       </x:c>
       <x:c r="B20" s="27" t="str">
         <x:v>待业务确认</x:v>
       </x:c>
-      <x:c r="C20" s="24" t="str">
+      <x:c r="C20" s="35" t="str">
         <x:v>若创建人只是录单人，不得用于个人复位评价</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="24" t="str">
         <x:v>轻度超配线</x:v>
       </x:c>
       <x:c r="B21" s="29" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="C21" s="24" t="str">
+      <x:c r="C21" s="35" t="str">
         <x:v>门店个人级升级版使用</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="24" t="str">
         <x:v>严重超配线</x:v>
       </x:c>
       <x:c r="B22" s="29" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="C22" s="24" t="str">
+      <x:c r="C22" s="35" t="str">
         <x:v>门店个人级升级版使用</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="24" t="str">
         <x:v>复位工资覆盖周末高峰</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
         <x:v>待业务确认</x:v>
       </x:c>
-      <x:c r="C23" s="24" t="str">
+      <x:c r="C23" s="35" t="str">
         <x:v>为“是”后，单波次人工成本才可用于经营判断</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
+    <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="25" t="str">
         <x:v>现有引流汇总已按目标日期过滤</x:v>
       </x:c>
       <x:c r="B24" s="28" t="str">
         <x:v>待业务确认</x:v>
       </x:c>
-      <x:c r="C24" s="25" t="str">
+      <x:c r="C24" s="36" t="str">
         <x:v>为“是”表示工时、成本、成交额只含周六、周日及国家法定节假日</x:v>
       </x:c>
     </x:row>
@@ -4989,26 +4989,26 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="7.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.440000057220459" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="10" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="28.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="32.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="6.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="10" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="8.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="8.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="22.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="24.440000534057617" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -5036,28 +5036,28 @@
       <x:c r="T1" s="4"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="37" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>本页只比较实际人工成本与成交金额。核心口径：每1元工资产生成交=引流成交金额÷引流实际人工成本；工时、成本和成交金额必须只覆盖周六、周日及国家法定节假日。</x:v>
       </x:c>
-      <x:c r="B2" s="37"/>
-      <x:c r="C2" s="37"/>
-      <x:c r="D2" s="37"/>
-      <x:c r="E2" s="37"/>
-      <x:c r="F2" s="37"/>
-      <x:c r="G2" s="37"/>
-      <x:c r="H2" s="37"/>
-      <x:c r="I2" s="37"/>
-      <x:c r="J2" s="37"/>
-      <x:c r="K2" s="37"/>
-      <x:c r="L2" s="37"/>
-      <x:c r="M2" s="37"/>
-      <x:c r="N2" s="37"/>
-      <x:c r="O2" s="37"/>
-      <x:c r="P2" s="37"/>
-      <x:c r="Q2" s="37"/>
-      <x:c r="R2" s="37"/>
-      <x:c r="S2" s="37"/>
-      <x:c r="T2" s="37"/>
+      <x:c r="B2" s="40"/>
+      <x:c r="C2" s="40"/>
+      <x:c r="D2" s="40"/>
+      <x:c r="E2" s="40"/>
+      <x:c r="F2" s="40"/>
+      <x:c r="G2" s="40"/>
+      <x:c r="H2" s="40"/>
+      <x:c r="I2" s="40"/>
+      <x:c r="J2" s="40"/>
+      <x:c r="K2" s="40"/>
+      <x:c r="L2" s="40"/>
+      <x:c r="M2" s="40"/>
+      <x:c r="N2" s="40"/>
+      <x:c r="O2" s="40"/>
+      <x:c r="P2" s="40"/>
+      <x:c r="Q2" s="40"/>
+      <x:c r="R2" s="40"/>
+      <x:c r="S2" s="40"/>
+      <x:c r="T2" s="40"/>
     </x:row>
     <x:row r="3" ht="34.5" customHeight="1">
       <x:c r="A3" s="16" t="str">
@@ -5121,7 +5121,7 @@
         <x:v>下周动作</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="31.5" customHeight="1">
       <x:c r="A4" s="23" t="str">
         <x:f>'门店周数据录入'!A4</x:f>
         <x:v>3区</x:v>
@@ -5190,16 +5190,16 @@
         <x:f>IF(OR(Q4="数据异常",Q4="人工数据缺失"),"待补数据",IF(OR(J4&lt;'规则参数'!$B$7,K4&lt;'规则参数'!$B$9),"引流低效",IF(OR(J4&lt;'规则参数'!$B$8,P4&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="S4" s="23" t="str">
+      <x:c r="S4" s="34" t="str">
         <x:f>IF(R4="待补数据","工时或成本口径不完整，先修正数据。",IF(J4&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K4&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P4&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>引流人工成本占门店营收偏高。</x:v>
       </x:c>
-      <x:c r="T4" s="23" t="str">
+      <x:c r="T4" s="34" t="str">
         <x:f>IF(R4="待补数据","补齐工时和实际成本后再判断。",IF(R4="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R4="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="31.5" customHeight="1">
       <x:c r="A5" s="24" t="str">
         <x:f>'门店周数据录入'!A5</x:f>
         <x:v>3区</x:v>
@@ -5268,16 +5268,16 @@
         <x:f>IF(OR(Q5="数据异常",Q5="人工数据缺失"),"待补数据",IF(OR(J5&lt;'规则参数'!$B$7,K5&lt;'规则参数'!$B$9),"引流低效",IF(OR(J5&lt;'规则参数'!$B$8,P5&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="S5" s="24" t="str">
+      <x:c r="S5" s="35" t="str">
         <x:f>IF(R5="待补数据","工时或成本口径不完整，先修正数据。",IF(J5&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K5&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P5&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>每小时成交金额偏低，先检查点位和时段。</x:v>
       </x:c>
-      <x:c r="T5" s="24" t="str">
+      <x:c r="T5" s="35" t="str">
         <x:f>IF(R5="待补数据","补齐工时和实际成本后再判断。",IF(R5="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R5="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="31.5" customHeight="1">
       <x:c r="A6" s="24" t="str">
         <x:f>'门店周数据录入'!A6</x:f>
         <x:v>1区</x:v>
@@ -5346,16 +5346,16 @@
         <x:f>IF(OR(Q6="数据异常",Q6="人工数据缺失"),"待补数据",IF(OR(J6&lt;'规则参数'!$B$7,K6&lt;'规则参数'!$B$9),"引流低效",IF(OR(J6&lt;'规则参数'!$B$8,P6&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="S6" s="24" t="str">
+      <x:c r="S6" s="35" t="str">
         <x:f>IF(R6="待补数据","工时或成本口径不完整，先修正数据。",IF(J6&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K6&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P6&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>每1元工资换回的成交金额低于低效线。</x:v>
       </x:c>
-      <x:c r="T6" s="24" t="str">
+      <x:c r="T6" s="35" t="str">
         <x:f>IF(R6="待补数据","补齐工时和实际成本后再判断。",IF(R6="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R6="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="31.5" customHeight="1">
       <x:c r="A7" s="24" t="str">
         <x:f>'门店周数据录入'!A7</x:f>
         <x:v>1区</x:v>
@@ -5424,16 +5424,16 @@
         <x:f>IF(OR(Q7="数据异常",Q7="人工数据缺失"),"待补数据",IF(OR(J7&lt;'规则参数'!$B$7,K7&lt;'规则参数'!$B$9),"引流低效",IF(OR(J7&lt;'规则参数'!$B$8,P7&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S7" s="24" t="str">
+      <x:c r="S7" s="35" t="str">
         <x:f>IF(R7="待补数据","工时或成本口径不完整，先修正数据。",IF(J7&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K7&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P7&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T7" s="24" t="str">
+      <x:c r="T7" s="35" t="str">
         <x:f>IF(R7="待补数据","补齐工时和实际成本后再判断。",IF(R7="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R7="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="31.5" customHeight="1">
       <x:c r="A8" s="24" t="str">
         <x:f>'门店周数据录入'!A8</x:f>
         <x:v>1区</x:v>
@@ -5502,16 +5502,16 @@
         <x:f>IF(OR(Q8="数据异常",Q8="人工数据缺失"),"待补数据",IF(OR(J8&lt;'规则参数'!$B$7,K8&lt;'规则参数'!$B$9),"引流低效",IF(OR(J8&lt;'规则参数'!$B$8,P8&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S8" s="24" t="str">
+      <x:c r="S8" s="35" t="str">
         <x:f>IF(R8="待补数据","工时或成本口径不完整，先修正数据。",IF(J8&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K8&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P8&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T8" s="24" t="str">
+      <x:c r="T8" s="35" t="str">
         <x:f>IF(R8="待补数据","补齐工时和实际成本后再判断。",IF(R8="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R8="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="31.5" customHeight="1">
       <x:c r="A9" s="24" t="str">
         <x:f>'门店周数据录入'!A9</x:f>
         <x:v>2区</x:v>
@@ -5580,16 +5580,16 @@
         <x:f>IF(OR(Q9="数据异常",Q9="人工数据缺失"),"待补数据",IF(OR(J9&lt;'规则参数'!$B$7,K9&lt;'规则参数'!$B$9),"引流低效",IF(OR(J9&lt;'规则参数'!$B$8,P9&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="S9" s="24" t="str">
+      <x:c r="S9" s="35" t="str">
         <x:f>IF(R9="待补数据","工时或成本口径不完整，先修正数据。",IF(J9&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K9&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P9&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>每小时成交金额偏低，先检查点位和时段。</x:v>
       </x:c>
-      <x:c r="T9" s="24" t="str">
+      <x:c r="T9" s="35" t="str">
         <x:f>IF(R9="待补数据","补齐工时和实际成本后再判断。",IF(R9="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R9="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="31.5" customHeight="1">
       <x:c r="A10" s="24" t="str">
         <x:f>'门店周数据录入'!A10</x:f>
         <x:v>1区</x:v>
@@ -5658,16 +5658,16 @@
         <x:f>IF(OR(Q10="数据异常",Q10="人工数据缺失"),"待补数据",IF(OR(J10&lt;'规则参数'!$B$7,K10&lt;'规则参数'!$B$9),"引流低效",IF(OR(J10&lt;'规则参数'!$B$8,P10&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="S10" s="24" t="str">
+      <x:c r="S10" s="35" t="str">
         <x:f>IF(R10="待补数据","工时或成本口径不完整，先修正数据。",IF(J10&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K10&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P10&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>引流人工成本占门店营收偏高。</x:v>
       </x:c>
-      <x:c r="T10" s="24" t="str">
+      <x:c r="T10" s="35" t="str">
         <x:f>IF(R10="待补数据","补齐工时和实际成本后再判断。",IF(R10="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R10="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="31.5" customHeight="1">
       <x:c r="A11" s="24" t="str">
         <x:f>'门店周数据录入'!A11</x:f>
         <x:v>3区</x:v>
@@ -5736,16 +5736,16 @@
         <x:f>IF(OR(Q11="数据异常",Q11="人工数据缺失"),"待补数据",IF(OR(J11&lt;'规则参数'!$B$7,K11&lt;'规则参数'!$B$9),"引流低效",IF(OR(J11&lt;'规则参数'!$B$8,P11&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S11" s="24" t="str">
+      <x:c r="S11" s="35" t="str">
         <x:f>IF(R11="待补数据","工时或成本口径不完整，先修正数据。",IF(J11&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K11&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P11&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T11" s="24" t="str">
+      <x:c r="T11" s="35" t="str">
         <x:f>IF(R11="待补数据","补齐工时和实际成本后再判断。",IF(R11="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R11="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="31.5" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:f>'门店周数据录入'!A12</x:f>
         <x:v>3区</x:v>
@@ -5814,16 +5814,16 @@
         <x:f>IF(OR(Q12="数据异常",Q12="人工数据缺失"),"待补数据",IF(OR(J12&lt;'规则参数'!$B$7,K12&lt;'规则参数'!$B$9),"引流低效",IF(OR(J12&lt;'规则参数'!$B$8,P12&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S12" s="24" t="str">
+      <x:c r="S12" s="35" t="str">
         <x:f>IF(R12="待补数据","工时或成本口径不完整，先修正数据。",IF(J12&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K12&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P12&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T12" s="24" t="str">
+      <x:c r="T12" s="35" t="str">
         <x:f>IF(R12="待补数据","补齐工时和实际成本后再判断。",IF(R12="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R12="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="31.5" customHeight="1">
       <x:c r="A13" s="24" t="str">
         <x:f>'门店周数据录入'!A13</x:f>
         <x:v>2区</x:v>
@@ -5892,16 +5892,16 @@
         <x:f>IF(OR(Q13="数据异常",Q13="人工数据缺失"),"待补数据",IF(OR(J13&lt;'规则参数'!$B$7,K13&lt;'规则参数'!$B$9),"引流低效",IF(OR(J13&lt;'规则参数'!$B$8,P13&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S13" s="24" t="str">
+      <x:c r="S13" s="35" t="str">
         <x:f>IF(R13="待补数据","工时或成本口径不完整，先修正数据。",IF(J13&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K13&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P13&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T13" s="24" t="str">
+      <x:c r="T13" s="35" t="str">
         <x:f>IF(R13="待补数据","补齐工时和实际成本后再判断。",IF(R13="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R13="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="31.5" customHeight="1">
       <x:c r="A14" s="24" t="str">
         <x:f>'门店周数据录入'!A14</x:f>
         <x:v>2区</x:v>
@@ -5970,16 +5970,16 @@
         <x:f>IF(OR(Q14="数据异常",Q14="人工数据缺失"),"待补数据",IF(OR(J14&lt;'规则参数'!$B$7,K14&lt;'规则参数'!$B$9),"引流低效",IF(OR(J14&lt;'规则参数'!$B$8,P14&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="S14" s="24" t="str">
+      <x:c r="S14" s="35" t="str">
         <x:f>IF(R14="待补数据","工时或成本口径不完整，先修正数据。",IF(J14&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K14&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P14&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>引流人工成本占门店营收偏高。</x:v>
       </x:c>
-      <x:c r="T14" s="24" t="str">
+      <x:c r="T14" s="35" t="str">
         <x:f>IF(R14="待补数据","补齐工时和实际成本后再判断。",IF(R14="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R14="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="31.5" customHeight="1">
       <x:c r="A15" s="24" t="str">
         <x:f>'门店周数据录入'!A15</x:f>
         <x:v>3区</x:v>
@@ -6048,16 +6048,16 @@
         <x:f>IF(OR(Q15="数据异常",Q15="人工数据缺失"),"待补数据",IF(OR(J15&lt;'规则参数'!$B$7,K15&lt;'规则参数'!$B$9),"引流低效",IF(OR(J15&lt;'规则参数'!$B$8,P15&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S15" s="24" t="str">
+      <x:c r="S15" s="35" t="str">
         <x:f>IF(R15="待补数据","工时或成本口径不完整，先修正数据。",IF(J15&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K15&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P15&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T15" s="24" t="str">
+      <x:c r="T15" s="35" t="str">
         <x:f>IF(R15="待补数据","补齐工时和实际成本后再判断。",IF(R15="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R15="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="31.5" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:f>'门店周数据录入'!A16</x:f>
         <x:v>2区</x:v>
@@ -6126,16 +6126,16 @@
         <x:f>IF(OR(Q16="数据异常",Q16="人工数据缺失"),"待补数据",IF(OR(J16&lt;'规则参数'!$B$7,K16&lt;'规则参数'!$B$9),"引流低效",IF(OR(J16&lt;'规则参数'!$B$8,P16&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S16" s="24" t="str">
+      <x:c r="S16" s="35" t="str">
         <x:f>IF(R16="待补数据","工时或成本口径不完整，先修正数据。",IF(J16&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K16&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P16&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T16" s="24" t="str">
+      <x:c r="T16" s="35" t="str">
         <x:f>IF(R16="待补数据","补齐工时和实际成本后再判断。",IF(R16="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R16="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="31.5" customHeight="1">
       <x:c r="A17" s="24" t="str">
         <x:f>'门店周数据录入'!A17</x:f>
         <x:v>2区</x:v>
@@ -6204,16 +6204,16 @@
         <x:f>IF(OR(Q17="数据异常",Q17="人工数据缺失"),"待补数据",IF(OR(J17&lt;'规则参数'!$B$7,K17&lt;'规则参数'!$B$9),"引流低效",IF(OR(J17&lt;'规则参数'!$B$8,P17&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S17" s="24" t="str">
+      <x:c r="S17" s="35" t="str">
         <x:f>IF(R17="待补数据","工时或成本口径不完整，先修正数据。",IF(J17&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K17&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P17&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T17" s="24" t="str">
+      <x:c r="T17" s="35" t="str">
         <x:f>IF(R17="待补数据","补齐工时和实际成本后再判断。",IF(R17="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R17="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="31.5" customHeight="1">
       <x:c r="A18" s="24" t="str">
         <x:f>'门店周数据录入'!A18</x:f>
         <x:v>3区</x:v>
@@ -6282,16 +6282,16 @@
         <x:f>IF(OR(Q18="数据异常",Q18="人工数据缺失"),"待补数据",IF(OR(J18&lt;'规则参数'!$B$7,K18&lt;'规则参数'!$B$9),"引流低效",IF(OR(J18&lt;'规则参数'!$B$8,P18&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流低效</x:v>
       </x:c>
-      <x:c r="S18" s="24" t="str">
+      <x:c r="S18" s="35" t="str">
         <x:f>IF(R18="待补数据","工时或成本口径不完整，先修正数据。",IF(J18&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K18&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P18&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>每1元工资换回的成交金额低于低效线。</x:v>
       </x:c>
-      <x:c r="T18" s="24" t="str">
+      <x:c r="T18" s="35" t="str">
         <x:f>IF(R18="待补数据","补齐工时和实际成本后再判断。",IF(R18="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R18="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>先减低效点位/时段工时，连续3周验证后再替换。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="31.5" customHeight="1">
       <x:c r="A19" s="24" t="str">
         <x:f>'门店周数据录入'!A19</x:f>
         <x:v>2区</x:v>
@@ -6360,16 +6360,16 @@
         <x:f>IF(OR(Q19="数据异常",Q19="人工数据缺失"),"待补数据",IF(OR(J19&lt;'规则参数'!$B$7,K19&lt;'规则参数'!$B$9),"引流低效",IF(OR(J19&lt;'规则参数'!$B$8,P19&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S19" s="24" t="str">
+      <x:c r="S19" s="35" t="str">
         <x:f>IF(R19="待补数据","工时或成本口径不完整，先修正数据。",IF(J19&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K19&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P19&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T19" s="24" t="str">
+      <x:c r="T19" s="35" t="str">
         <x:f>IF(R19="待补数据","补齐工时和实际成本后再判断。",IF(R19="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R19="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="31.5" customHeight="1">
       <x:c r="A20" s="24" t="str">
         <x:f>'门店周数据录入'!A20</x:f>
         <x:v>1区</x:v>
@@ -6438,16 +6438,16 @@
         <x:f>IF(OR(Q20="数据异常",Q20="人工数据缺失"),"待补数据",IF(OR(J20&lt;'规则参数'!$B$7,K20&lt;'规则参数'!$B$9),"引流低效",IF(OR(J20&lt;'规则参数'!$B$8,P20&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S20" s="24" t="str">
+      <x:c r="S20" s="35" t="str">
         <x:f>IF(R20="待补数据","工时或成本口径不完整，先修正数据。",IF(J20&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K20&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P20&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T20" s="24" t="str">
+      <x:c r="T20" s="35" t="str">
         <x:f>IF(R20="待补数据","补齐工时和实际成本后再判断。",IF(R20="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R20="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="31.5" customHeight="1">
       <x:c r="A21" s="24" t="str">
         <x:f>'门店周数据录入'!A21</x:f>
         <x:v>1区</x:v>
@@ -6516,16 +6516,16 @@
         <x:f>IF(OR(Q21="数据异常",Q21="人工数据缺失"),"待补数据",IF(OR(J21&lt;'规则参数'!$B$7,K21&lt;'规则参数'!$B$9),"引流低效",IF(OR(J21&lt;'规则参数'!$B$8,P21&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流优秀</x:v>
       </x:c>
-      <x:c r="S21" s="24" t="str">
+      <x:c r="S21" s="35" t="str">
         <x:f>IF(R21="待补数据","工时或成本口径不完整，先修正数据。",IF(J21&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K21&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P21&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>产出倍数与小时产出均达标。</x:v>
       </x:c>
-      <x:c r="T21" s="24" t="str">
+      <x:c r="T21" s="35" t="str">
         <x:f>IF(R21="待补数据","补齐工时和实际成本后再判断。",IF(R21="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R21="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>保持或增加有效点位排班，并培养复制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="31.5" customHeight="1">
       <x:c r="A22" s="25" t="str">
         <x:f>'门店周数据录入'!A22</x:f>
         <x:v>2区</x:v>
@@ -6594,11 +6594,11 @@
         <x:f>IF(OR(Q22="数据异常",Q22="人工数据缺失"),"待补数据",IF(OR(J22&lt;'规则参数'!$B$7,K22&lt;'规则参数'!$B$9),"引流低效",IF(OR(J22&lt;'规则参数'!$B$8,P22&gt;'规则参数'!$B$10),"引流观察","引流优秀")))</x:f>
         <x:v>引流观察</x:v>
       </x:c>
-      <x:c r="S22" s="25" t="str">
+      <x:c r="S22" s="36" t="str">
         <x:f>IF(R22="待补数据","工时或成本口径不完整，先修正数据。",IF(J22&lt;'规则参数'!$B$7,"每1元工资换回的成交金额低于低效线。",IF(K22&lt;'规则参数'!$B$9,"每小时成交金额偏低，先检查点位和时段。",IF(P22&gt;'规则参数'!$B$10,"引流人工成本占门店营收偏高。","产出倍数与小时产出均达标。"))))</x:f>
         <x:v>引流人工成本占门店营收偏高。</x:v>
       </x:c>
-      <x:c r="T22" s="25" t="str">
+      <x:c r="T22" s="36" t="str">
         <x:f>IF(R22="待补数据","补齐工时和实际成本后再判断。",IF(R22="引流低效","先减低效点位/时段工时，连续3周验证后再替换。",IF(R22="引流观察","调整点位与时段，下一周复盘。","保持或增加有效点位排班，并培养复制。")))</x:f>
         <x:v>调整点位与时段，下一周复盘。</x:v>
       </x:c>
@@ -6627,7 +6627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R518a43053dc54723"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45ffe436e1684260"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6636,23 +6636,23 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="7.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.440000057220459" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="28.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="33.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="6.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="6.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="9.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -6677,25 +6677,25 @@
       <x:c r="Q1" s="4"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="37" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>实际波次/人/时按两天12小时计算。源表“复位工资”周期尚未证明只覆盖周末高峰；确认前，单波次人工成本仅作提示，不参与复位紧松判断。</x:v>
       </x:c>
-      <x:c r="B2" s="37"/>
-      <x:c r="C2" s="37"/>
-      <x:c r="D2" s="37"/>
-      <x:c r="E2" s="37"/>
-      <x:c r="F2" s="37"/>
-      <x:c r="G2" s="37"/>
-      <x:c r="H2" s="37"/>
-      <x:c r="I2" s="37"/>
-      <x:c r="J2" s="37"/>
-      <x:c r="K2" s="37"/>
-      <x:c r="L2" s="37"/>
-      <x:c r="M2" s="37"/>
-      <x:c r="N2" s="37"/>
-      <x:c r="O2" s="37"/>
-      <x:c r="P2" s="37"/>
-      <x:c r="Q2" s="37"/>
+      <x:c r="B2" s="40"/>
+      <x:c r="C2" s="40"/>
+      <x:c r="D2" s="40"/>
+      <x:c r="E2" s="40"/>
+      <x:c r="F2" s="40"/>
+      <x:c r="G2" s="40"/>
+      <x:c r="H2" s="40"/>
+      <x:c r="I2" s="40"/>
+      <x:c r="J2" s="40"/>
+      <x:c r="K2" s="40"/>
+      <x:c r="L2" s="40"/>
+      <x:c r="M2" s="40"/>
+      <x:c r="N2" s="40"/>
+      <x:c r="O2" s="40"/>
+      <x:c r="P2" s="40"/>
+      <x:c r="Q2" s="40"/>
     </x:row>
     <x:row r="3" ht="34.5" customHeight="1">
       <x:c r="A3" s="16" t="str">
@@ -6750,7 +6750,7 @@
         <x:v>下周动作</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="33" customHeight="1">
       <x:c r="A4" s="23" t="str">
         <x:f>'门店周数据录入'!A4</x:f>
         <x:v>3区</x:v>
@@ -6811,16 +6811,16 @@
         <x:f>IF(OR(E4&lt;=0,F4&lt;=0),"数据异常",IF(OR(K4&gt;='规则参数'!$B$16,L4&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H4&gt;'规则参数'!$B$12,J4&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H4&lt;'规则参数'!$B$11,K4&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P4" s="23" t="str">
+      <x:c r="P4" s="34" t="str">
         <x:f>IF(O4="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O4="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O4="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O4="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q4" s="23" t="str">
+      <x:c r="Q4" s="34" t="str">
         <x:f>IF(O4="数据异常","先补齐或核实人数、波次和成本。",IF(O4="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O4="结构偏紧","观察两周并准备高峰机动支援。",IF(O4="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="33" customHeight="1">
       <x:c r="A5" s="24" t="str">
         <x:f>'门店周数据录入'!A5</x:f>
         <x:v>3区</x:v>
@@ -6881,16 +6881,16 @@
         <x:f>IF(OR(E5&lt;=0,F5&lt;=0),"数据异常",IF(OR(K5&gt;='规则参数'!$B$16,L5&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H5&gt;'规则参数'!$B$12,J5&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H5&lt;'规则参数'!$B$11,K5&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>复位偏松</x:v>
       </x:c>
-      <x:c r="P5" s="24" t="str">
+      <x:c r="P5" s="35" t="str">
         <x:f>IF(O5="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O5="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O5="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O5="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>结构负荷与实际波次同时偏低，可能存在工时浪费。</x:v>
       </x:c>
-      <x:c r="Q5" s="24" t="str">
+      <x:c r="Q5" s="35" t="str">
         <x:f>IF(O5="数据异常","先补齐或核实人数、波次和成本。",IF(O5="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O5="结构偏紧","观察两周并准备高峰机动支援。",IF(O5="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>先减低峰工时，再减低效工时；连续3周后才替换。</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="33" customHeight="1">
       <x:c r="A6" s="24" t="str">
         <x:f>'门店周数据录入'!A6</x:f>
         <x:v>1区</x:v>
@@ -6951,16 +6951,16 @@
         <x:f>IF(OR(E6&lt;=0,F6&lt;=0),"数据异常",IF(OR(K6&gt;='规则参数'!$B$16,L6&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H6&gt;'规则参数'!$B$12,J6&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H6&lt;'规则参数'!$B$11,K6&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P6" s="24" t="str">
+      <x:c r="P6" s="35" t="str">
         <x:f>IF(O6="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O6="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O6="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O6="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q6" s="24" t="str">
+      <x:c r="Q6" s="35" t="str">
         <x:f>IF(O6="数据异常","先补齐或核实人数、波次和成本。",IF(O6="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O6="结构偏紧","观察两周并准备高峰机动支援。",IF(O6="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="33" customHeight="1">
       <x:c r="A7" s="24" t="str">
         <x:f>'门店周数据录入'!A7</x:f>
         <x:v>1区</x:v>
@@ -7021,16 +7021,16 @@
         <x:f>IF(OR(E7&lt;=0,F7&lt;=0),"数据异常",IF(OR(K7&gt;='规则参数'!$B$16,L7&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H7&gt;'规则参数'!$B$12,J7&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H7&lt;'规则参数'!$B$11,K7&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P7" s="24" t="str">
+      <x:c r="P7" s="35" t="str">
         <x:f>IF(O7="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O7="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O7="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O7="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q7" s="24" t="str">
+      <x:c r="Q7" s="35" t="str">
         <x:f>IF(O7="数据异常","先补齐或核实人数、波次和成本。",IF(O7="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O7="结构偏紧","观察两周并准备高峰机动支援。",IF(O7="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="33" customHeight="1">
       <x:c r="A8" s="24" t="str">
         <x:f>'门店周数据录入'!A8</x:f>
         <x:v>1区</x:v>
@@ -7091,16 +7091,16 @@
         <x:f>IF(OR(E8&lt;=0,F8&lt;=0),"数据异常",IF(OR(K8&gt;='规则参数'!$B$16,L8&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H8&gt;'规则参数'!$B$12,J8&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H8&lt;'规则参数'!$B$11,K8&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P8" s="24" t="str">
+      <x:c r="P8" s="35" t="str">
         <x:f>IF(O8="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O8="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O8="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O8="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q8" s="24" t="str">
+      <x:c r="Q8" s="35" t="str">
         <x:f>IF(O8="数据异常","先补齐或核实人数、波次和成本。",IF(O8="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O8="结构偏紧","观察两周并准备高峰机动支援。",IF(O8="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="33" customHeight="1">
       <x:c r="A9" s="24" t="str">
         <x:f>'门店周数据录入'!A9</x:f>
         <x:v>2区</x:v>
@@ -7161,16 +7161,16 @@
         <x:f>IF(OR(E9&lt;=0,F9&lt;=0),"数据异常",IF(OR(K9&gt;='规则参数'!$B$16,L9&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H9&gt;'规则参数'!$B$12,J9&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H9&lt;'规则参数'!$B$11,K9&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>高峰偏紧</x:v>
       </x:c>
-      <x:c r="P9" s="24" t="str">
+      <x:c r="P9" s="35" t="str">
         <x:f>IF(O9="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O9="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O9="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O9="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>两天高峰实际承接强度或理论利用率过高。</x:v>
       </x:c>
-      <x:c r="Q9" s="24" t="str">
+      <x:c r="Q9" s="35" t="str">
         <x:f>IF(O9="数据异常","先补齐或核实人数、波次和成本。",IF(O9="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O9="结构偏紧","观察两周并准备高峰机动支援。",IF(O9="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>增加高峰支持或错峰排班，避免服务风险。</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="33" customHeight="1">
       <x:c r="A10" s="24" t="str">
         <x:f>'门店周数据录入'!A10</x:f>
         <x:v>1区</x:v>
@@ -7231,16 +7231,16 @@
         <x:f>IF(OR(E10&lt;=0,F10&lt;=0),"数据异常",IF(OR(K10&gt;='规则参数'!$B$16,L10&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H10&gt;'规则参数'!$B$12,J10&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H10&lt;'规则参数'!$B$11,K10&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P10" s="24" t="str">
+      <x:c r="P10" s="35" t="str">
         <x:f>IF(O10="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O10="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O10="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O10="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q10" s="24" t="str">
+      <x:c r="Q10" s="35" t="str">
         <x:f>IF(O10="数据异常","先补齐或核实人数、波次和成本。",IF(O10="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O10="结构偏紧","观察两周并准备高峰机动支援。",IF(O10="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="33" customHeight="1">
       <x:c r="A11" s="24" t="str">
         <x:f>'门店周数据录入'!A11</x:f>
         <x:v>3区</x:v>
@@ -7301,16 +7301,16 @@
         <x:f>IF(OR(E11&lt;=0,F11&lt;=0),"数据异常",IF(OR(K11&gt;='规则参数'!$B$16,L11&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H11&gt;'规则参数'!$B$12,J11&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H11&lt;'规则参数'!$B$11,K11&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P11" s="24" t="str">
+      <x:c r="P11" s="35" t="str">
         <x:f>IF(O11="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O11="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O11="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O11="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q11" s="24" t="str">
+      <x:c r="Q11" s="35" t="str">
         <x:f>IF(O11="数据异常","先补齐或核实人数、波次和成本。",IF(O11="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O11="结构偏紧","观察两周并准备高峰机动支援。",IF(O11="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="33" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:f>'门店周数据录入'!A12</x:f>
         <x:v>3区</x:v>
@@ -7371,16 +7371,16 @@
         <x:f>IF(OR(E12&lt;=0,F12&lt;=0),"数据异常",IF(OR(K12&gt;='规则参数'!$B$16,L12&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H12&gt;'规则参数'!$B$12,J12&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H12&lt;'规则参数'!$B$11,K12&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P12" s="24" t="str">
+      <x:c r="P12" s="35" t="str">
         <x:f>IF(O12="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O12="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O12="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O12="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q12" s="24" t="str">
+      <x:c r="Q12" s="35" t="str">
         <x:f>IF(O12="数据异常","先补齐或核实人数、波次和成本。",IF(O12="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O12="结构偏紧","观察两周并准备高峰机动支援。",IF(O12="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="33" customHeight="1">
       <x:c r="A13" s="24" t="str">
         <x:f>'门店周数据录入'!A13</x:f>
         <x:v>2区</x:v>
@@ -7441,16 +7441,16 @@
         <x:f>IF(OR(E13&lt;=0,F13&lt;=0),"数据异常",IF(OR(K13&gt;='规则参数'!$B$16,L13&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H13&gt;'规则参数'!$B$12,J13&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H13&lt;'规则参数'!$B$11,K13&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P13" s="24" t="str">
+      <x:c r="P13" s="35" t="str">
         <x:f>IF(O13="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O13="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O13="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O13="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q13" s="24" t="str">
+      <x:c r="Q13" s="35" t="str">
         <x:f>IF(O13="数据异常","先补齐或核实人数、波次和成本。",IF(O13="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O13="结构偏紧","观察两周并准备高峰机动支援。",IF(O13="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="33" customHeight="1">
       <x:c r="A14" s="24" t="str">
         <x:f>'门店周数据录入'!A14</x:f>
         <x:v>2区</x:v>
@@ -7511,16 +7511,16 @@
         <x:f>IF(OR(E14&lt;=0,F14&lt;=0),"数据异常",IF(OR(K14&gt;='规则参数'!$B$16,L14&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H14&gt;'规则参数'!$B$12,J14&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H14&lt;'规则参数'!$B$11,K14&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P14" s="24" t="str">
+      <x:c r="P14" s="35" t="str">
         <x:f>IF(O14="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O14="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O14="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O14="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q14" s="24" t="str">
+      <x:c r="Q14" s="35" t="str">
         <x:f>IF(O14="数据异常","先补齐或核实人数、波次和成本。",IF(O14="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O14="结构偏紧","观察两周并准备高峰机动支援。",IF(O14="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="33" customHeight="1">
       <x:c r="A15" s="24" t="str">
         <x:f>'门店周数据录入'!A15</x:f>
         <x:v>3区</x:v>
@@ -7581,16 +7581,16 @@
         <x:f>IF(OR(E15&lt;=0,F15&lt;=0),"数据异常",IF(OR(K15&gt;='规则参数'!$B$16,L15&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H15&gt;'规则参数'!$B$12,J15&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H15&lt;'规则参数'!$B$11,K15&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P15" s="24" t="str">
+      <x:c r="P15" s="35" t="str">
         <x:f>IF(O15="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O15="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O15="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O15="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q15" s="24" t="str">
+      <x:c r="Q15" s="35" t="str">
         <x:f>IF(O15="数据异常","先补齐或核实人数、波次和成本。",IF(O15="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O15="结构偏紧","观察两周并准备高峰机动支援。",IF(O15="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="33" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:f>'门店周数据录入'!A16</x:f>
         <x:v>2区</x:v>
@@ -7651,16 +7651,16 @@
         <x:f>IF(OR(E16&lt;=0,F16&lt;=0),"数据异常",IF(OR(K16&gt;='规则参数'!$B$16,L16&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H16&gt;'规则参数'!$B$12,J16&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H16&lt;'规则参数'!$B$11,K16&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>高峰偏紧</x:v>
       </x:c>
-      <x:c r="P16" s="24" t="str">
+      <x:c r="P16" s="35" t="str">
         <x:f>IF(O16="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O16="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O16="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O16="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>两天高峰实际承接强度或理论利用率过高。</x:v>
       </x:c>
-      <x:c r="Q16" s="24" t="str">
+      <x:c r="Q16" s="35" t="str">
         <x:f>IF(O16="数据异常","先补齐或核实人数、波次和成本。",IF(O16="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O16="结构偏紧","观察两周并准备高峰机动支援。",IF(O16="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>增加高峰支持或错峰排班，避免服务风险。</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="33" customHeight="1">
       <x:c r="A17" s="24" t="str">
         <x:f>'门店周数据录入'!A17</x:f>
         <x:v>2区</x:v>
@@ -7721,16 +7721,16 @@
         <x:f>IF(OR(E17&lt;=0,F17&lt;=0),"数据异常",IF(OR(K17&gt;='规则参数'!$B$16,L17&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H17&gt;'规则参数'!$B$12,J17&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H17&lt;'规则参数'!$B$11,K17&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P17" s="24" t="str">
+      <x:c r="P17" s="35" t="str">
         <x:f>IF(O17="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O17="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O17="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O17="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q17" s="24" t="str">
+      <x:c r="Q17" s="35" t="str">
         <x:f>IF(O17="数据异常","先补齐或核实人数、波次和成本。",IF(O17="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O17="结构偏紧","观察两周并准备高峰机动支援。",IF(O17="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="33" customHeight="1">
       <x:c r="A18" s="24" t="str">
         <x:f>'门店周数据录入'!A18</x:f>
         <x:v>3区</x:v>
@@ -7791,16 +7791,16 @@
         <x:f>IF(OR(E18&lt;=0,F18&lt;=0),"数据异常",IF(OR(K18&gt;='规则参数'!$B$16,L18&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H18&gt;'规则参数'!$B$12,J18&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H18&lt;'规则参数'!$B$11,K18&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P18" s="24" t="str">
+      <x:c r="P18" s="35" t="str">
         <x:f>IF(O18="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O18="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O18="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O18="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q18" s="24" t="str">
+      <x:c r="Q18" s="35" t="str">
         <x:f>IF(O18="数据异常","先补齐或核实人数、波次和成本。",IF(O18="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O18="结构偏紧","观察两周并准备高峰机动支援。",IF(O18="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="33" customHeight="1">
       <x:c r="A19" s="24" t="str">
         <x:f>'门店周数据录入'!A19</x:f>
         <x:v>2区</x:v>
@@ -7861,16 +7861,16 @@
         <x:f>IF(OR(E19&lt;=0,F19&lt;=0),"数据异常",IF(OR(K19&gt;='规则参数'!$B$16,L19&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H19&gt;'规则参数'!$B$12,J19&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H19&lt;'规则参数'!$B$11,K19&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P19" s="24" t="str">
+      <x:c r="P19" s="35" t="str">
         <x:f>IF(O19="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O19="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O19="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O19="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q19" s="24" t="str">
+      <x:c r="Q19" s="35" t="str">
         <x:f>IF(O19="数据异常","先补齐或核实人数、波次和成本。",IF(O19="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O19="结构偏紧","观察两周并准备高峰机动支援。",IF(O19="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="33" customHeight="1">
       <x:c r="A20" s="24" t="str">
         <x:f>'门店周数据录入'!A20</x:f>
         <x:v>1区</x:v>
@@ -7931,16 +7931,16 @@
         <x:f>IF(OR(E20&lt;=0,F20&lt;=0),"数据异常",IF(OR(K20&gt;='规则参数'!$B$16,L20&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H20&gt;'规则参数'!$B$12,J20&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H20&lt;'规则参数'!$B$11,K20&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P20" s="24" t="str">
+      <x:c r="P20" s="35" t="str">
         <x:f>IF(O20="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O20="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O20="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O20="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q20" s="24" t="str">
+      <x:c r="Q20" s="35" t="str">
         <x:f>IF(O20="数据异常","先补齐或核实人数、波次和成本。",IF(O20="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O20="结构偏紧","观察两周并准备高峰机动支援。",IF(O20="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="33" customHeight="1">
       <x:c r="A21" s="24" t="str">
         <x:f>'门店周数据录入'!A21</x:f>
         <x:v>1区</x:v>
@@ -7998,16 +7998,16 @@
         <x:f>IF(OR(E21&lt;=0,F21&lt;=0),"数据异常",IF(OR(K21&gt;='规则参数'!$B$16,L21&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H21&gt;'规则参数'!$B$12,J21&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H21&lt;'规则参数'!$B$11,K21&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>数据异常</x:v>
       </x:c>
-      <x:c r="P21" s="24" t="str">
+      <x:c r="P21" s="35" t="str">
         <x:f>IF(O21="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O21="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O21="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O21="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>人数、波次或成本不完整，不能评价配置。</x:v>
       </x:c>
-      <x:c r="Q21" s="24" t="str">
+      <x:c r="Q21" s="35" t="str">
         <x:f>IF(O21="数据异常","先补齐或核实人数、波次和成本。",IF(O21="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O21="结构偏紧","观察两周并准备高峰机动支援。",IF(O21="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>先补齐或核实人数、波次和成本。</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="33" customHeight="1">
       <x:c r="A22" s="25" t="str">
         <x:f>'门店周数据录入'!A22</x:f>
         <x:v>2区</x:v>
@@ -8068,11 +8068,11 @@
         <x:f>IF(OR(E22&lt;=0,F22&lt;=0),"数据异常",IF(OR(K22&gt;='规则参数'!$B$16,L22&gt;='规则参数'!$B$17),"高峰偏紧",IF(OR(H22&gt;'规则参数'!$B$12,J22&gt;'规则参数'!$B$14),"结构偏紧",IF(AND(H22&lt;'规则参数'!$B$11,K22&lt;'规则参数'!$B$15),"复位偏松","配置合理"))))</x:f>
         <x:v>配置合理</x:v>
       </x:c>
-      <x:c r="P22" s="25" t="str">
+      <x:c r="P22" s="36" t="str">
         <x:f>IF(O22="数据异常","人数、波次或成本不完整，不能评价配置。",IF(O22="高峰偏紧","两天高峰实际承接强度或理论利用率过高。",IF(O22="结构偏紧","单人负责主题过多，需防止高峰服务风险。",IF(O22="复位偏松","结构负荷与实际波次同时偏低，可能存在工时浪费。","实际承接与结构负荷处于合理区间。"))))</x:f>
         <x:v>实际承接与结构负荷处于合理区间。</x:v>
       </x:c>
-      <x:c r="Q22" s="25" t="str">
+      <x:c r="Q22" s="36" t="str">
         <x:f>IF(O22="数据异常","先补齐或核实人数、波次和成本。",IF(O22="高峰偏紧","增加高峰支持或错峰排班，避免服务风险。",IF(O22="结构偏紧","观察两周并准备高峰机动支援。",IF(O22="复位偏松","先减低峰工时，再减低效工时；连续3周后才替换。","保持配置，继续周度跟踪。"))))</x:f>
         <x:v>保持配置，继续周度跟踪。</x:v>
       </x:c>
@@ -8101,7 +8101,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31cdef1401f94cbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R751d8beaebc54b27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8110,21 +8110,21 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="7.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="9.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="9.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="28.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="10" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="9.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="42.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="6.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="8.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="8.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="8.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="8.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="8.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="8" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="28.889999389648438" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -8147,23 +8147,23 @@
       <x:c r="O1" s="4"/>
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
-      <x:c r="A2" s="37" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>CHECK不等于经营差，表示仍有字段缺失或口径需确认；ERROR表示当前数据会直接导致计算错误或严重误判。引流成交金额大于门店总营收，可能因包含充值或跨期归属，需业务确认但不自动判错。</x:v>
       </x:c>
-      <x:c r="B2" s="37"/>
-      <x:c r="C2" s="37"/>
-      <x:c r="D2" s="37"/>
-      <x:c r="E2" s="37"/>
-      <x:c r="F2" s="37"/>
-      <x:c r="G2" s="37"/>
-      <x:c r="H2" s="37"/>
-      <x:c r="I2" s="37"/>
-      <x:c r="J2" s="37"/>
-      <x:c r="K2" s="37"/>
-      <x:c r="L2" s="37"/>
-      <x:c r="M2" s="37"/>
-      <x:c r="N2" s="37"/>
-      <x:c r="O2" s="37"/>
+      <x:c r="B2" s="40"/>
+      <x:c r="C2" s="40"/>
+      <x:c r="D2" s="40"/>
+      <x:c r="E2" s="40"/>
+      <x:c r="F2" s="40"/>
+      <x:c r="G2" s="40"/>
+      <x:c r="H2" s="40"/>
+      <x:c r="I2" s="40"/>
+      <x:c r="J2" s="40"/>
+      <x:c r="K2" s="40"/>
+      <x:c r="L2" s="40"/>
+      <x:c r="M2" s="40"/>
+      <x:c r="N2" s="40"/>
+      <x:c r="O2" s="40"/>
     </x:row>
     <x:row r="3" ht="34.5" customHeight="1">
       <x:c r="A3" s="16" t="str">
@@ -8269,9 +8269,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O4&gt;0,C4&lt;=0),AND(K4&gt;0,J4&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F4&lt;&gt;"已填",G4&lt;&gt;"已填",I4&lt;&gt;"正常",M4&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O4" s="38" t="str">
-        <x:f>IF(N4="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F4="缺失","补填引流到店人数；","")&amp;IF(G4="缺失","补填办卡数；","")&amp;IF(I4&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M4&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O4" s="34" t="str">
+        <x:f>IF(N4="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F4="缺失","补到店；","")&amp;IF(G4="缺失","补办卡；","")&amp;IF(I4&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M4&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="33" customHeight="1">
@@ -8331,9 +8331,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O5&gt;0,C5&lt;=0),AND(K5&gt;0,J5&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F5&lt;&gt;"已填",G5&lt;&gt;"已填",I5&lt;&gt;"正常",M5&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O5" s="39" t="str">
-        <x:f>IF(N5="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F5="缺失","补填引流到店人数；","")&amp;IF(G5="缺失","补填办卡数；","")&amp;IF(I5&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M5&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O5" s="35" t="str">
+        <x:f>IF(N5="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F5="缺失","补到店；","")&amp;IF(G5="缺失","补办卡；","")&amp;IF(I5&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M5&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="33" customHeight="1">
@@ -8393,9 +8393,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O6&gt;0,C6&lt;=0),AND(K6&gt;0,J6&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F6&lt;&gt;"已填",G6&lt;&gt;"已填",I6&lt;&gt;"正常",M6&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O6" s="39" t="str">
-        <x:f>IF(N6="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F6="缺失","补填引流到店人数；","")&amp;IF(G6="缺失","补填办卡数；","")&amp;IF(I6&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M6&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O6" s="35" t="str">
+        <x:f>IF(N6="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F6="缺失","补到店；","")&amp;IF(G6="缺失","补办卡；","")&amp;IF(I6&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M6&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="33" customHeight="1">
@@ -8455,9 +8455,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O7&gt;0,C7&lt;=0),AND(K7&gt;0,J7&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F7&lt;&gt;"已填",G7&lt;&gt;"已填",I7&lt;&gt;"正常",M7&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O7" s="39" t="str">
-        <x:f>IF(N7="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F7="缺失","补填引流到店人数；","")&amp;IF(G7="缺失","补填办卡数；","")&amp;IF(I7&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M7&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O7" s="35" t="str">
+        <x:f>IF(N7="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F7="缺失","补到店；","")&amp;IF(G7="缺失","补办卡；","")&amp;IF(I7&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M7&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="33" customHeight="1">
@@ -8517,9 +8517,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O8&gt;0,C8&lt;=0),AND(K8&gt;0,J8&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F8&lt;&gt;"已填",G8&lt;&gt;"已填",I8&lt;&gt;"正常",M8&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O8" s="39" t="str">
-        <x:f>IF(N8="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F8="缺失","补填引流到店人数；","")&amp;IF(G8="缺失","补填办卡数；","")&amp;IF(I8&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M8&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O8" s="35" t="str">
+        <x:f>IF(N8="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F8="缺失","补到店；","")&amp;IF(G8="缺失","补办卡；","")&amp;IF(I8&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M8&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="33" customHeight="1">
@@ -8579,9 +8579,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O9&gt;0,C9&lt;=0),AND(K9&gt;0,J9&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F9&lt;&gt;"已填",G9&lt;&gt;"已填",I9&lt;&gt;"正常",M9&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O9" s="39" t="str">
-        <x:f>IF(N9="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F9="缺失","补填引流到店人数；","")&amp;IF(G9="缺失","补填办卡数；","")&amp;IF(I9&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M9&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O9" s="35" t="str">
+        <x:f>IF(N9="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F9="缺失","补到店；","")&amp;IF(G9="缺失","补办卡；","")&amp;IF(I9&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M9&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="33" customHeight="1">
@@ -8641,9 +8641,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O10&gt;0,C10&lt;=0),AND(K10&gt;0,J10&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F10&lt;&gt;"已填",G10&lt;&gt;"已填",I10&lt;&gt;"正常",M10&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O10" s="39" t="str">
-        <x:f>IF(N10="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F10="缺失","补填引流到店人数；","")&amp;IF(G10="缺失","补填办卡数；","")&amp;IF(I10&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M10&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认成交金额是否含充值/跨期；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O10" s="35" t="str">
+        <x:f>IF(N10="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F10="缺失","补到店；","")&amp;IF(G10="缺失","补办卡；","")&amp;IF(I10&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M10&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对成交额范围；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="33" customHeight="1">
@@ -8703,9 +8703,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O11&gt;0,C11&lt;=0),AND(K11&gt;0,J11&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F11&lt;&gt;"已填",G11&lt;&gt;"已填",I11&lt;&gt;"正常",M11&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O11" s="39" t="str">
-        <x:f>IF(N11="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F11="缺失","补填引流到店人数；","")&amp;IF(G11="缺失","补填办卡数；","")&amp;IF(I11&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M11&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认成交金额是否含充值/跨期；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O11" s="35" t="str">
+        <x:f>IF(N11="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F11="缺失","补到店；","")&amp;IF(G11="缺失","补办卡；","")&amp;IF(I11&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M11&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对成交额范围；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="33" customHeight="1">
@@ -8765,9 +8765,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O12&gt;0,C12&lt;=0),AND(K12&gt;0,J12&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F12&lt;&gt;"已填",G12&lt;&gt;"已填",I12&lt;&gt;"正常",M12&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O12" s="39" t="str">
-        <x:f>IF(N12="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F12="缺失","补填引流到店人数；","")&amp;IF(G12="缺失","补填办卡数；","")&amp;IF(I12&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M12&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O12" s="35" t="str">
+        <x:f>IF(N12="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F12="缺失","补到店；","")&amp;IF(G12="缺失","补办卡；","")&amp;IF(I12&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M12&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="33" customHeight="1">
@@ -8827,9 +8827,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O13&gt;0,C13&lt;=0),AND(K13&gt;0,J13&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F13&lt;&gt;"已填",G13&lt;&gt;"已填",I13&lt;&gt;"正常",M13&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O13" s="39" t="str">
-        <x:f>IF(N13="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F13="缺失","补填引流到店人数；","")&amp;IF(G13="缺失","补填办卡数；","")&amp;IF(I13&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M13&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O13" s="35" t="str">
+        <x:f>IF(N13="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F13="缺失","补到店；","")&amp;IF(G13="缺失","补办卡；","")&amp;IF(I13&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M13&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="33" customHeight="1">
@@ -8889,9 +8889,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O14&gt;0,C14&lt;=0),AND(K14&gt;0,J14&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F14&lt;&gt;"已填",G14&lt;&gt;"已填",I14&lt;&gt;"正常",M14&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O14" s="39" t="str">
-        <x:f>IF(N14="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F14="缺失","补填引流到店人数；","")&amp;IF(G14="缺失","补填办卡数；","")&amp;IF(I14&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M14&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认成交金额是否含充值/跨期；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O14" s="35" t="str">
+        <x:f>IF(N14="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F14="缺失","补到店；","")&amp;IF(G14="缺失","补办卡；","")&amp;IF(I14&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M14&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对成交额范围；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="33" customHeight="1">
@@ -8951,9 +8951,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O15&gt;0,C15&lt;=0),AND(K15&gt;0,J15&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F15&lt;&gt;"已填",G15&lt;&gt;"已填",I15&lt;&gt;"正常",M15&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O15" s="39" t="str">
-        <x:f>IF(N15="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F15="缺失","补填引流到店人数；","")&amp;IF(G15="缺失","补填办卡数；","")&amp;IF(I15&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M15&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认成交金额是否含充值/跨期；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O15" s="35" t="str">
+        <x:f>IF(N15="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F15="缺失","补到店；","")&amp;IF(G15="缺失","补办卡；","")&amp;IF(I15&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M15&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对成交额范围；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="33" customHeight="1">
@@ -9013,9 +9013,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O16&gt;0,C16&lt;=0),AND(K16&gt;0,J16&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F16&lt;&gt;"已填",G16&lt;&gt;"已填",I16&lt;&gt;"正常",M16&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O16" s="39" t="str">
-        <x:f>IF(N16="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F16="缺失","补填引流到店人数；","")&amp;IF(G16="缺失","补填办卡数；","")&amp;IF(I16&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M16&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O16" s="35" t="str">
+        <x:f>IF(N16="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F16="缺失","补到店；","")&amp;IF(G16="缺失","补办卡；","")&amp;IF(I16&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M16&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="33" customHeight="1">
@@ -9075,9 +9075,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O17&gt;0,C17&lt;=0),AND(K17&gt;0,J17&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F17&lt;&gt;"已填",G17&lt;&gt;"已填",I17&lt;&gt;"正常",M17&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O17" s="39" t="str">
-        <x:f>IF(N17="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F17="缺失","补填引流到店人数；","")&amp;IF(G17="缺失","补填办卡数；","")&amp;IF(I17&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M17&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O17" s="35" t="str">
+        <x:f>IF(N17="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F17="缺失","补到店；","")&amp;IF(G17="缺失","补办卡；","")&amp;IF(I17&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M17&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
@@ -9137,9 +9137,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O18&gt;0,C18&lt;=0),AND(K18&gt;0,J18&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F18&lt;&gt;"已填",G18&lt;&gt;"已填",I18&lt;&gt;"正常",M18&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O18" s="39" t="str">
-        <x:f>IF(N18="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F18="缺失","补填引流到店人数；","")&amp;IF(G18="缺失","补填办卡数；","")&amp;IF(I18&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M18&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O18" s="35" t="str">
+        <x:f>IF(N18="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F18="缺失","补到店；","")&amp;IF(G18="缺失","补办卡；","")&amp;IF(I18&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M18&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="33" customHeight="1">
@@ -9199,9 +9199,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O19&gt;0,C19&lt;=0),AND(K19&gt;0,J19&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F19&lt;&gt;"已填",G19&lt;&gt;"已填",I19&lt;&gt;"正常",M19&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O19" s="39" t="str">
-        <x:f>IF(N19="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F19="缺失","补填引流到店人数；","")&amp;IF(G19="缺失","补填办卡数；","")&amp;IF(I19&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M19&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O19" s="35" t="str">
+        <x:f>IF(N19="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F19="缺失","补到店；","")&amp;IF(G19="缺失","补办卡；","")&amp;IF(I19&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M19&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="33" customHeight="1">
@@ -9261,9 +9261,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O20&gt;0,C20&lt;=0),AND(K20&gt;0,J20&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F20&lt;&gt;"已填",G20&lt;&gt;"已填",I20&lt;&gt;"正常",M20&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O20" s="39" t="str">
-        <x:f>IF(N20="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F20="缺失","补填引流到店人数；","")&amp;IF(G20="缺失","补填办卡数；","")&amp;IF(I20&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M20&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O20" s="35" t="str">
+        <x:f>IF(N20="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F20="缺失","补到店；","")&amp;IF(G20="缺失","补办卡；","")&amp;IF(I20&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M20&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="33" customHeight="1">
@@ -9323,9 +9323,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O21&gt;0,C21&lt;=0),AND(K21&gt;0,J21&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F21&lt;&gt;"已填",G21&lt;&gt;"已填",I21&lt;&gt;"正常",M21&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>ERROR</x:v>
       </x:c>
-      <x:c r="O21" s="39" t="str">
-        <x:f>IF(N21="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F21="缺失","补填引流到店人数；","")&amp;IF(G21="缺失","补填办卡数；","")&amp;IF(I21&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M21&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>立即修正人数、工时或成本，不得用于判断。</x:v>
+      <x:c r="O21" s="35" t="str">
+        <x:f>IF(N21="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F21="缺失","补到店；","")&amp;IF(G21="缺失","补办卡；","")&amp;IF(I21&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M21&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>修正人数、工时或成本，暂停判断。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="33" customHeight="1">
@@ -9385,9 +9385,9 @@
         <x:f>IF(OR(AND('门店周数据录入'!O22&gt;0,C22&lt;=0),AND(K22&gt;0,J22&lt;=0)),"ERROR",IF(OR('规则参数'!$B$24&lt;&gt;"是",F22&lt;&gt;"已填",G22&lt;&gt;"已填",I22&lt;&gt;"正常",M22&lt;&gt;"完整"),"CHECK","PASS"))</x:f>
         <x:v>CHECK</x:v>
       </x:c>
-      <x:c r="O22" s="40" t="str">
-        <x:f>IF(N22="ERROR","立即修正人数、工时或成本，不得用于判断。",IF('规则参数'!$B$24&lt;&gt;"是","确认引流数据仅含周末/国家法定节假日；","")&amp;IF(F22="缺失","补填引流到店人数；","")&amp;IF(G22="缺失","补填办卡数；","")&amp;IF(I22&lt;&gt;"正常","确认成交金额是否含充值/跨期；","")&amp;IF(M22&lt;&gt;"完整","确认复位工资是否覆盖周末高峰；",""))</x:f>
-        <x:v>确认引流数据仅含周末/国家法定节假日；补填引流到店人数；补填办卡数；确认成交金额是否含充值/跨期；确认复位工资是否覆盖周末高峰；</x:v>
+      <x:c r="O22" s="36" t="str">
+        <x:f>IF(N22="ERROR","修正人数、工时或成本，暂停判断。",IF('规则参数'!$B$24&lt;&gt;"是","核对引流日期；","")&amp;IF(F22="缺失","补到店；","")&amp;IF(G22="缺失","补办卡；","")&amp;IF(I22&lt;&gt;"正常","核对成交额范围；","")&amp;IF(M22&lt;&gt;"完整","核对复位工资周期；",""))</x:f>
+        <x:v>核对引流日期；补到店；补办卡；核对成交额范围；核对复位工资周期；</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9414,7 +9414,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f3667636a348c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95a167c2b040487c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9423,23 +9423,23 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="10" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="9.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="10" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="8.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22.219999313354492" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -9464,25 +9464,25 @@
       <x:c r="Q1" s="4"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="36" t="str">
+      <x:c r="A2" s="39" t="str">
         <x:v>每个周六、周日和国家法定节假日每天一行；黄色列由店长填写。引流实际成本=工时×实际时薪+额外提成/奖励。复位字段只填周六、周日14:00-20:00；唯一账单ID计1个房间波次。空白=未填，0=确认没有。</x:v>
       </x:c>
-      <x:c r="B2" s="36"/>
-      <x:c r="C2" s="36"/>
-      <x:c r="D2" s="36"/>
-      <x:c r="E2" s="36"/>
-      <x:c r="F2" s="36"/>
-      <x:c r="G2" s="36"/>
-      <x:c r="H2" s="36"/>
-      <x:c r="I2" s="36"/>
-      <x:c r="J2" s="36"/>
-      <x:c r="K2" s="36"/>
-      <x:c r="L2" s="36"/>
-      <x:c r="M2" s="36"/>
-      <x:c r="N2" s="36"/>
-      <x:c r="O2" s="36"/>
-      <x:c r="P2" s="36"/>
-      <x:c r="Q2" s="36"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
+      <x:c r="F2" s="39"/>
+      <x:c r="G2" s="39"/>
+      <x:c r="H2" s="39"/>
+      <x:c r="I2" s="39"/>
+      <x:c r="J2" s="39"/>
+      <x:c r="K2" s="39"/>
+      <x:c r="L2" s="39"/>
+      <x:c r="M2" s="39"/>
+      <x:c r="N2" s="39"/>
+      <x:c r="O2" s="39"/>
+      <x:c r="P2" s="39"/>
+      <x:c r="Q2" s="39"/>
     </x:row>
     <x:row r="3" ht="34.5" customHeight="1">
       <x:c r="A3" s="16" t="str">
@@ -9537,7 +9537,7 @@
         <x:v>备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="22.5" customHeight="1">
       <x:c r="A4" s="100"/>
       <x:c r="B4" s="26"/>
       <x:c r="C4" s="26"/>
@@ -9556,9 +9556,9 @@
       <x:c r="N4" s="47"/>
       <x:c r="O4" s="47"/>
       <x:c r="P4" s="47"/>
-      <x:c r="Q4" s="26"/>
-    </x:row>
-    <x:row r="5">
+      <x:c r="Q4" s="41"/>
+    </x:row>
+    <x:row r="5" ht="22.5" customHeight="1">
       <x:c r="A5" s="101"/>
       <x:c r="B5" s="27"/>
       <x:c r="C5" s="27"/>
@@ -9577,9 +9577,9 @@
       <x:c r="N5" s="48"/>
       <x:c r="O5" s="48"/>
       <x:c r="P5" s="48"/>
-      <x:c r="Q5" s="27"/>
-    </x:row>
-    <x:row r="6">
+      <x:c r="Q5" s="42"/>
+    </x:row>
+    <x:row r="6" ht="22.5" customHeight="1">
       <x:c r="A6" s="101"/>
       <x:c r="B6" s="27"/>
       <x:c r="C6" s="27"/>
@@ -9598,9 +9598,9 @@
       <x:c r="N6" s="48"/>
       <x:c r="O6" s="48"/>
       <x:c r="P6" s="48"/>
-      <x:c r="Q6" s="27"/>
-    </x:row>
-    <x:row r="7">
+      <x:c r="Q6" s="42"/>
+    </x:row>
+    <x:row r="7" ht="22.5" customHeight="1">
       <x:c r="A7" s="101"/>
       <x:c r="B7" s="27"/>
       <x:c r="C7" s="27"/>
@@ -9619,9 +9619,9 @@
       <x:c r="N7" s="48"/>
       <x:c r="O7" s="48"/>
       <x:c r="P7" s="48"/>
-      <x:c r="Q7" s="27"/>
-    </x:row>
-    <x:row r="8">
+      <x:c r="Q7" s="42"/>
+    </x:row>
+    <x:row r="8" ht="22.5" customHeight="1">
       <x:c r="A8" s="101"/>
       <x:c r="B8" s="27"/>
       <x:c r="C8" s="27"/>
@@ -9640,9 +9640,9 @@
       <x:c r="N8" s="48"/>
       <x:c r="O8" s="48"/>
       <x:c r="P8" s="48"/>
-      <x:c r="Q8" s="27"/>
-    </x:row>
-    <x:row r="9">
+      <x:c r="Q8" s="42"/>
+    </x:row>
+    <x:row r="9" ht="22.5" customHeight="1">
       <x:c r="A9" s="101"/>
       <x:c r="B9" s="27"/>
       <x:c r="C9" s="27"/>
@@ -9661,9 +9661,9 @@
       <x:c r="N9" s="48"/>
       <x:c r="O9" s="48"/>
       <x:c r="P9" s="48"/>
-      <x:c r="Q9" s="27"/>
-    </x:row>
-    <x:row r="10">
+      <x:c r="Q9" s="42"/>
+    </x:row>
+    <x:row r="10" ht="22.5" customHeight="1">
       <x:c r="A10" s="101"/>
       <x:c r="B10" s="27"/>
       <x:c r="C10" s="27"/>
@@ -9682,9 +9682,9 @@
       <x:c r="N10" s="48"/>
       <x:c r="O10" s="48"/>
       <x:c r="P10" s="48"/>
-      <x:c r="Q10" s="27"/>
-    </x:row>
-    <x:row r="11">
+      <x:c r="Q10" s="42"/>
+    </x:row>
+    <x:row r="11" ht="22.5" customHeight="1">
       <x:c r="A11" s="101"/>
       <x:c r="B11" s="27"/>
       <x:c r="C11" s="27"/>
@@ -9703,9 +9703,9 @@
       <x:c r="N11" s="48"/>
       <x:c r="O11" s="48"/>
       <x:c r="P11" s="48"/>
-      <x:c r="Q11" s="27"/>
-    </x:row>
-    <x:row r="12">
+      <x:c r="Q11" s="42"/>
+    </x:row>
+    <x:row r="12" ht="22.5" customHeight="1">
       <x:c r="A12" s="101"/>
       <x:c r="B12" s="27"/>
       <x:c r="C12" s="27"/>
@@ -9724,9 +9724,9 @@
       <x:c r="N12" s="48"/>
       <x:c r="O12" s="48"/>
       <x:c r="P12" s="48"/>
-      <x:c r="Q12" s="27"/>
-    </x:row>
-    <x:row r="13">
+      <x:c r="Q12" s="42"/>
+    </x:row>
+    <x:row r="13" ht="22.5" customHeight="1">
       <x:c r="A13" s="101"/>
       <x:c r="B13" s="27"/>
       <x:c r="C13" s="27"/>
@@ -9745,9 +9745,9 @@
       <x:c r="N13" s="48"/>
       <x:c r="O13" s="48"/>
       <x:c r="P13" s="48"/>
-      <x:c r="Q13" s="27"/>
-    </x:row>
-    <x:row r="14">
+      <x:c r="Q13" s="42"/>
+    </x:row>
+    <x:row r="14" ht="22.5" customHeight="1">
       <x:c r="A14" s="101"/>
       <x:c r="B14" s="27"/>
       <x:c r="C14" s="27"/>
@@ -9766,9 +9766,9 @@
       <x:c r="N14" s="48"/>
       <x:c r="O14" s="48"/>
       <x:c r="P14" s="48"/>
-      <x:c r="Q14" s="27"/>
-    </x:row>
-    <x:row r="15">
+      <x:c r="Q14" s="42"/>
+    </x:row>
+    <x:row r="15" ht="22.5" customHeight="1">
       <x:c r="A15" s="101"/>
       <x:c r="B15" s="27"/>
       <x:c r="C15" s="27"/>
@@ -9787,9 +9787,9 @@
       <x:c r="N15" s="48"/>
       <x:c r="O15" s="48"/>
       <x:c r="P15" s="48"/>
-      <x:c r="Q15" s="27"/>
-    </x:row>
-    <x:row r="16">
+      <x:c r="Q15" s="42"/>
+    </x:row>
+    <x:row r="16" ht="22.5" customHeight="1">
       <x:c r="A16" s="101"/>
       <x:c r="B16" s="27"/>
       <x:c r="C16" s="27"/>
@@ -9808,9 +9808,9 @@
       <x:c r="N16" s="48"/>
       <x:c r="O16" s="48"/>
       <x:c r="P16" s="48"/>
-      <x:c r="Q16" s="27"/>
-    </x:row>
-    <x:row r="17">
+      <x:c r="Q16" s="42"/>
+    </x:row>
+    <x:row r="17" ht="22.5" customHeight="1">
       <x:c r="A17" s="101"/>
       <x:c r="B17" s="27"/>
       <x:c r="C17" s="27"/>
@@ -9829,9 +9829,9 @@
       <x:c r="N17" s="48"/>
       <x:c r="O17" s="48"/>
       <x:c r="P17" s="48"/>
-      <x:c r="Q17" s="27"/>
-    </x:row>
-    <x:row r="18">
+      <x:c r="Q17" s="42"/>
+    </x:row>
+    <x:row r="18" ht="22.5" customHeight="1">
       <x:c r="A18" s="101"/>
       <x:c r="B18" s="27"/>
       <x:c r="C18" s="27"/>
@@ -9850,9 +9850,9 @@
       <x:c r="N18" s="48"/>
       <x:c r="O18" s="48"/>
       <x:c r="P18" s="48"/>
-      <x:c r="Q18" s="27"/>
-    </x:row>
-    <x:row r="19">
+      <x:c r="Q18" s="42"/>
+    </x:row>
+    <x:row r="19" ht="22.5" customHeight="1">
       <x:c r="A19" s="101"/>
       <x:c r="B19" s="27"/>
       <x:c r="C19" s="27"/>
@@ -9871,9 +9871,9 @@
       <x:c r="N19" s="48"/>
       <x:c r="O19" s="48"/>
       <x:c r="P19" s="48"/>
-      <x:c r="Q19" s="27"/>
-    </x:row>
-    <x:row r="20">
+      <x:c r="Q19" s="42"/>
+    </x:row>
+    <x:row r="20" ht="22.5" customHeight="1">
       <x:c r="A20" s="101"/>
       <x:c r="B20" s="27"/>
       <x:c r="C20" s="27"/>
@@ -9892,9 +9892,9 @@
       <x:c r="N20" s="48"/>
       <x:c r="O20" s="48"/>
       <x:c r="P20" s="48"/>
-      <x:c r="Q20" s="27"/>
-    </x:row>
-    <x:row r="21">
+      <x:c r="Q20" s="42"/>
+    </x:row>
+    <x:row r="21" ht="22.5" customHeight="1">
       <x:c r="A21" s="101"/>
       <x:c r="B21" s="27"/>
       <x:c r="C21" s="27"/>
@@ -9913,9 +9913,9 @@
       <x:c r="N21" s="48"/>
       <x:c r="O21" s="48"/>
       <x:c r="P21" s="48"/>
-      <x:c r="Q21" s="27"/>
-    </x:row>
-    <x:row r="22">
+      <x:c r="Q21" s="42"/>
+    </x:row>
+    <x:row r="22" ht="22.5" customHeight="1">
       <x:c r="A22" s="101"/>
       <x:c r="B22" s="27"/>
       <x:c r="C22" s="27"/>
@@ -9934,9 +9934,9 @@
       <x:c r="N22" s="48"/>
       <x:c r="O22" s="48"/>
       <x:c r="P22" s="48"/>
-      <x:c r="Q22" s="27"/>
-    </x:row>
-    <x:row r="23">
+      <x:c r="Q22" s="42"/>
+    </x:row>
+    <x:row r="23" ht="22.5" customHeight="1">
       <x:c r="A23" s="101"/>
       <x:c r="B23" s="27"/>
       <x:c r="C23" s="27"/>
@@ -9955,9 +9955,9 @@
       <x:c r="N23" s="48"/>
       <x:c r="O23" s="48"/>
       <x:c r="P23" s="48"/>
-      <x:c r="Q23" s="27"/>
-    </x:row>
-    <x:row r="24">
+      <x:c r="Q23" s="42"/>
+    </x:row>
+    <x:row r="24" ht="22.5" customHeight="1">
       <x:c r="A24" s="101"/>
       <x:c r="B24" s="27"/>
       <x:c r="C24" s="27"/>
@@ -9976,9 +9976,9 @@
       <x:c r="N24" s="48"/>
       <x:c r="O24" s="48"/>
       <x:c r="P24" s="48"/>
-      <x:c r="Q24" s="27"/>
-    </x:row>
-    <x:row r="25">
+      <x:c r="Q24" s="42"/>
+    </x:row>
+    <x:row r="25" ht="22.5" customHeight="1">
       <x:c r="A25" s="101"/>
       <x:c r="B25" s="27"/>
       <x:c r="C25" s="27"/>
@@ -9997,9 +9997,9 @@
       <x:c r="N25" s="48"/>
       <x:c r="O25" s="48"/>
       <x:c r="P25" s="48"/>
-      <x:c r="Q25" s="27"/>
-    </x:row>
-    <x:row r="26">
+      <x:c r="Q25" s="42"/>
+    </x:row>
+    <x:row r="26" ht="22.5" customHeight="1">
       <x:c r="A26" s="101"/>
       <x:c r="B26" s="27"/>
       <x:c r="C26" s="27"/>
@@ -10018,9 +10018,9 @@
       <x:c r="N26" s="48"/>
       <x:c r="O26" s="48"/>
       <x:c r="P26" s="48"/>
-      <x:c r="Q26" s="27"/>
-    </x:row>
-    <x:row r="27">
+      <x:c r="Q26" s="42"/>
+    </x:row>
+    <x:row r="27" ht="22.5" customHeight="1">
       <x:c r="A27" s="101"/>
       <x:c r="B27" s="27"/>
       <x:c r="C27" s="27"/>
@@ -10039,9 +10039,9 @@
       <x:c r="N27" s="48"/>
       <x:c r="O27" s="48"/>
       <x:c r="P27" s="48"/>
-      <x:c r="Q27" s="27"/>
-    </x:row>
-    <x:row r="28">
+      <x:c r="Q27" s="42"/>
+    </x:row>
+    <x:row r="28" ht="22.5" customHeight="1">
       <x:c r="A28" s="101"/>
       <x:c r="B28" s="27"/>
       <x:c r="C28" s="27"/>
@@ -10060,9 +10060,9 @@
       <x:c r="N28" s="48"/>
       <x:c r="O28" s="48"/>
       <x:c r="P28" s="48"/>
-      <x:c r="Q28" s="27"/>
-    </x:row>
-    <x:row r="29">
+      <x:c r="Q28" s="42"/>
+    </x:row>
+    <x:row r="29" ht="22.5" customHeight="1">
       <x:c r="A29" s="101"/>
       <x:c r="B29" s="27"/>
       <x:c r="C29" s="27"/>
@@ -10081,9 +10081,9 @@
       <x:c r="N29" s="48"/>
       <x:c r="O29" s="48"/>
       <x:c r="P29" s="48"/>
-      <x:c r="Q29" s="27"/>
-    </x:row>
-    <x:row r="30">
+      <x:c r="Q29" s="42"/>
+    </x:row>
+    <x:row r="30" ht="22.5" customHeight="1">
       <x:c r="A30" s="101"/>
       <x:c r="B30" s="27"/>
       <x:c r="C30" s="27"/>
@@ -10102,9 +10102,9 @@
       <x:c r="N30" s="48"/>
       <x:c r="O30" s="48"/>
       <x:c r="P30" s="48"/>
-      <x:c r="Q30" s="27"/>
-    </x:row>
-    <x:row r="31">
+      <x:c r="Q30" s="42"/>
+    </x:row>
+    <x:row r="31" ht="22.5" customHeight="1">
       <x:c r="A31" s="101"/>
       <x:c r="B31" s="27"/>
       <x:c r="C31" s="27"/>
@@ -10123,9 +10123,9 @@
       <x:c r="N31" s="48"/>
       <x:c r="O31" s="48"/>
       <x:c r="P31" s="48"/>
-      <x:c r="Q31" s="27"/>
-    </x:row>
-    <x:row r="32">
+      <x:c r="Q31" s="42"/>
+    </x:row>
+    <x:row r="32" ht="22.5" customHeight="1">
       <x:c r="A32" s="101"/>
       <x:c r="B32" s="27"/>
       <x:c r="C32" s="27"/>
@@ -10144,9 +10144,9 @@
       <x:c r="N32" s="48"/>
       <x:c r="O32" s="48"/>
       <x:c r="P32" s="48"/>
-      <x:c r="Q32" s="27"/>
-    </x:row>
-    <x:row r="33">
+      <x:c r="Q32" s="42"/>
+    </x:row>
+    <x:row r="33" ht="22.5" customHeight="1">
       <x:c r="A33" s="101"/>
       <x:c r="B33" s="27"/>
       <x:c r="C33" s="27"/>
@@ -10165,9 +10165,9 @@
       <x:c r="N33" s="48"/>
       <x:c r="O33" s="48"/>
       <x:c r="P33" s="48"/>
-      <x:c r="Q33" s="27"/>
-    </x:row>
-    <x:row r="34">
+      <x:c r="Q33" s="42"/>
+    </x:row>
+    <x:row r="34" ht="22.5" customHeight="1">
       <x:c r="A34" s="101"/>
       <x:c r="B34" s="27"/>
       <x:c r="C34" s="27"/>
@@ -10186,9 +10186,9 @@
       <x:c r="N34" s="48"/>
       <x:c r="O34" s="48"/>
       <x:c r="P34" s="48"/>
-      <x:c r="Q34" s="27"/>
-    </x:row>
-    <x:row r="35">
+      <x:c r="Q34" s="42"/>
+    </x:row>
+    <x:row r="35" ht="22.5" customHeight="1">
       <x:c r="A35" s="102"/>
       <x:c r="B35" s="28"/>
       <x:c r="C35" s="28"/>
@@ -10207,7 +10207,7 @@
       <x:c r="N35" s="49"/>
       <x:c r="O35" s="49"/>
       <x:c r="P35" s="49"/>
-      <x:c r="Q35" s="28"/>
+      <x:c r="Q35" s="43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -10224,7 +10224,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45c2ee508e64464f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8664c33d811e44f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10233,10 +10233,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="46.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="46.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="42.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="37.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="37.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35.560001373291016" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -10262,212 +10262,212 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
-      <x:c r="A4" s="38" t="str">
+      <x:c r="A4" s="34" t="str">
         <x:v>引流产出倍数</x:v>
       </x:c>
-      <x:c r="B4" s="38" t="str">
+      <x:c r="B4" s="34" t="str">
         <x:v>成交金额÷实际人工成本</x:v>
       </x:c>
-      <x:c r="C4" s="38" t="str">
+      <x:c r="C4" s="34" t="str">
         <x:v>回答1元工资换回多少成交额</x:v>
       </x:c>
-      <x:c r="D4" s="38" t="str">
+      <x:c r="D4" s="34" t="str">
         <x:v>只反映工资与成交额的关系</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="39" t="str">
+      <x:c r="A5" s="35" t="str">
         <x:v>双成本</x:v>
       </x:c>
-      <x:c r="B5" s="39" t="str">
+      <x:c r="B5" s="35" t="str">
         <x:v>标准成本=工时×10；实际成本按实发成本</x:v>
       </x:c>
-      <x:c r="C5" s="39" t="str">
+      <x:c r="C5" s="35" t="str">
         <x:v>横向排名用标准成本，经营判断用实际成本</x:v>
       </x:c>
-      <x:c r="D5" s="39" t="str">
+      <x:c r="D5" s="35" t="str">
         <x:v>节假日12-15元、提成和奖励必须进入实际成本</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
-      <x:c r="A6" s="39" t="str">
+      <x:c r="A6" s="35" t="str">
         <x:v>引流周期</x:v>
       </x:c>
-      <x:c r="B6" s="39" t="str">
+      <x:c r="B6" s="35" t="str">
         <x:v>每周六、周日及国家法定节假日</x:v>
       </x:c>
-      <x:c r="C6" s="39" t="str">
+      <x:c r="C6" s="35" t="str">
         <x:v>工时、成本、成交额必须只取这些日期</x:v>
       </x:c>
-      <x:c r="D6" s="39" t="str">
+      <x:c r="D6" s="35" t="str">
         <x:v>混入普通工作日会扭曲人效</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
-      <x:c r="A7" s="39" t="str">
+      <x:c r="A7" s="35" t="str">
         <x:v>复位周期</x:v>
       </x:c>
-      <x:c r="B7" s="39" t="str">
+      <x:c r="B7" s="35" t="str">
         <x:v>周六+周日14:00-20:00，共12小时</x:v>
       </x:c>
-      <x:c r="C7" s="39" t="str">
+      <x:c r="C7" s="35" t="str">
         <x:v>人数使用两天单日平均；波次为两天合计</x:v>
       </x:c>
-      <x:c r="D7" s="39" t="str">
+      <x:c r="D7" s="35" t="str">
         <x:v>原版只除6小时，会把实际人效放大一倍</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
-      <x:c r="A8" s="39" t="str">
+      <x:c r="A8" s="35" t="str">
         <x:v>房间波次</x:v>
       </x:c>
-      <x:c r="B8" s="39" t="str">
+      <x:c r="B8" s="35" t="str">
         <x:v>一个唯一账单ID=一个房间波次</x:v>
       </x:c>
-      <x:c r="C8" s="39" t="str">
+      <x:c r="C8" s="35" t="str">
         <x:v>禁止用玩家人数代替房间数</x:v>
       </x:c>
-      <x:c r="D8" s="39" t="str">
+      <x:c r="D8" s="35" t="str">
         <x:v>重复账单ID必须先去重</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
-      <x:c r="A9" s="39" t="str">
+      <x:c r="A9" s="35" t="str">
         <x:v>实际波次/人/时</x:v>
       </x:c>
-      <x:c r="B9" s="39" t="str">
+      <x:c r="B9" s="35" t="str">
         <x:v>两天高峰唯一账单数÷平均复位人数÷12小时</x:v>
       </x:c>
-      <x:c r="C9" s="39" t="str">
+      <x:c r="C9" s="35" t="str">
         <x:v>用于判断真实高峰承接压力</x:v>
       </x:c>
-      <x:c r="D9" s="39" t="str">
+      <x:c r="D9" s="35" t="str">
         <x:v>人数为0但波次&gt;0属于数据异常</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="36" customHeight="1">
-      <x:c r="A10" s="39" t="str">
+      <x:c r="A10" s="35" t="str">
         <x:v>理论最大波次</x:v>
       </x:c>
-      <x:c r="B10" s="39" t="str">
+      <x:c r="B10" s="35" t="str">
         <x:v>主题数×12小时×60÷40分钟</x:v>
       </x:c>
-      <x:c r="C10" s="39" t="str">
+      <x:c r="C10" s="35" t="str">
         <x:v>只作为利用率上限和结构风险参考</x:v>
       </x:c>
-      <x:c r="D10" s="39" t="str">
+      <x:c r="D10" s="35" t="str">
         <x:v>不等于真实应该完成的目标</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
-      <x:c r="A11" s="39" t="str">
+      <x:c r="A11" s="35" t="str">
         <x:v>复位评价</x:v>
       </x:c>
-      <x:c r="B11" s="39" t="str">
+      <x:c r="B11" s="35" t="str">
         <x:v>不使用门店营收ROI</x:v>
       </x:c>
-      <x:c r="C11" s="39" t="str">
+      <x:c r="C11" s="35" t="str">
         <x:v>看实际承接、主题负荷、利用率和单波次成本</x:v>
       </x:c>
-      <x:c r="D11" s="39" t="str">
+      <x:c r="D11" s="35" t="str">
         <x:v>创建人是否为实际接待负责人仍待业务确认</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
-      <x:c r="A12" s="39" t="str">
+      <x:c r="A12" s="35" t="str">
         <x:v>缺失值</x:v>
       </x:c>
-      <x:c r="B12" s="39" t="str">
+      <x:c r="B12" s="35" t="str">
         <x:v>空白=缺失；0=业务确认确实为0</x:v>
       </x:c>
-      <x:c r="C12" s="39" t="str">
+      <x:c r="C12" s="35" t="str">
         <x:v>先补数再评价，CHECK不等于经营差</x:v>
       </x:c>
-      <x:c r="D12" s="39" t="str">
+      <x:c r="D12" s="35" t="str">
         <x:v>原表到店、办卡占位0已改为空白</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
-      <x:c r="A13" s="39" t="str">
+      <x:c r="A13" s="35" t="str">
         <x:v>成交额范围</x:v>
       </x:c>
-      <x:c r="B13" s="39" t="str">
+      <x:c r="B13" s="35" t="str">
         <x:v>若引流成交额&gt;门店总营收，标记口径确认</x:v>
       </x:c>
-      <x:c r="C13" s="39" t="str">
+      <x:c r="C13" s="35" t="str">
         <x:v>可能含充值、跨期或跨门店归属</x:v>
       </x:c>
-      <x:c r="D13" s="39" t="str">
+      <x:c r="D13" s="35" t="str">
         <x:v>不自动删数，也不自动判错</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
-      <x:c r="A14" s="39" t="str">
+      <x:c r="A14" s="35" t="str">
         <x:v>老板动作顺序</x:v>
       </x:c>
-      <x:c r="B14" s="39" t="str">
+      <x:c r="B14" s="35" t="str">
         <x:v>补数据→减低峰工时→减低效工时→调岗位→连续3周验证后替换</x:v>
       </x:c>
-      <x:c r="C14" s="39" t="str">
+      <x:c r="C14" s="35" t="str">
         <x:v>禁止单周直接淘汰</x:v>
       </x:c>
-      <x:c r="D14" s="39" t="str">
+      <x:c r="D14" s="35" t="str">
         <x:v>至少连续3周看趋势</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
-      <x:c r="A15" s="39" t="str">
+      <x:c r="A15" s="35" t="str">
         <x:v>当前模型层级</x:v>
       </x:c>
-      <x:c r="B15" s="39" t="str">
+      <x:c r="B15" s="35" t="str">
         <x:v>门店级、岗位级</x:v>
       </x:c>
-      <x:c r="C15" s="39" t="str">
+      <x:c r="C15" s="35" t="str">
         <x:v>用于发现引流效率和复位高峰配置问题</x:v>
       </x:c>
-      <x:c r="D15" s="39" t="str">
+      <x:c r="D15" s="35" t="str">
         <x:v>不能回答具体哪位兼职应增排/减排</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="36" customHeight="1">
-      <x:c r="A16" s="39" t="str">
+      <x:c r="A16" s="35" t="str">
         <x:v>个人级升级所需</x:v>
       </x:c>
-      <x:c r="B16" s="39" t="str">
+      <x:c r="B16" s="35" t="str">
         <x:v>人员ID、姓名、每日工时、岗位、实际成本、成交归属、唯一账单创建归属</x:v>
       </x:c>
-      <x:c r="C16" s="39" t="str">
+      <x:c r="C16" s="35" t="str">
         <x:v>支持暑假工主岗位+副岗位和两周人员变化</x:v>
       </x:c>
-      <x:c r="D16" s="39" t="str">
+      <x:c r="D16" s="35" t="str">
         <x:v>同名人员必须用人员ID去重</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="36" customHeight="1">
-      <x:c r="A17" s="39" t="str">
+      <x:c r="A17" s="35" t="str">
         <x:v>门店超配升级所需</x:v>
       </x:c>
-      <x:c r="B17" s="39" t="str">
+      <x:c r="B17" s="35" t="str">
         <x:v>全职实际高峰覆盖工时、兼职实际工时、建议支持工时</x:v>
       </x:c>
-      <x:c r="C17" s="39" t="str">
+      <x:c r="C17" s="35" t="str">
         <x:v>超配工时=实际兼职工时-建议兼职工时</x:v>
       </x:c>
-      <x:c r="D17" s="39" t="str">
+      <x:c r="D17" s="35" t="str">
         <x:v>当前源表缺少全职覆盖和复位工时，不能可靠输出超配率</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
-      <x:c r="A18" s="40" t="str">
+      <x:c r="A18" s="36" t="str">
         <x:v>数据来源</x:v>
       </x:c>
-      <x:c r="B18" s="40" t="str">
+      <x:c r="B18" s="36" t="str">
         <x:v>老板确认版Excel；门店周报；唯一账单ID统计</x:v>
       </x:c>
-      <x:c r="C18" s="40" t="str">
+      <x:c r="C18" s="36" t="str">
         <x:v>所有输入均集中在“门店周数据录入”</x:v>
       </x:c>
-      <x:c r="D18" s="40" t="str">
+      <x:c r="D18" s="36" t="str">
         <x:v>现有汇总值与飞书周末日明细不一致，使用前必须确认日期过滤</x:v>
       </x:c>
     </x:row>

</xml_diff>